<commit_message>
market mapping 2026-09-16 — correction anti-doublons hospitality (Le Burgundy -> Hotel L'Ormaie) + rebuild XLSX/rapport
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013SpNGhZy6Aq6Bw2dFszH4M
</commit_message>
<xml_diff>
--- a/outputs/humanup_market_mapping_2026-09-16.xlsx
+++ b/outputs/humanup_market_mapping_2026-09-16.xlsx
@@ -2708,12 +2708,12 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Directeur General de l'hotel</t>
+          <t>Directeur de l'hotel</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Le Burgundy Paris</t>
+          <t>Hotel L'Ormaie</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -2729,12 +2729,12 @@
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>HOSPITALITY,JOB,DIRECTEUR_HOTEL,50-200,CONTACT_1,CONTACT_NON_SOURCE</t>
+          <t>HOSPITALITY,JOB,DIRECTEUR_HOTEL,5-50,CONTACT_1,CONTACT_NON_SOURCE</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Poste: Concierge (CDI) | Date: NC | Effectif: NC (hotel 5* independant, 59 chambres) | CA: NC | Salaire: NC | Source: Journal des Palaces | Lien: https://www.journaldespalaces.com/carriere/offre-318382-Concierge-Le-Burgundy-Paris.html | Contexte: Hotel 5* parisien independant (rue Duphot, Paris 1er). Recrutement d'un concierge en CDI, offre la plus recente du flux Journal des Palaces consultee.</t>
+          <t>Poste: Chef de reception (CDI) | Date: NC - offre active, ID 316727 (anteriorite probable &gt; 7 jours, a revalider) | Effectif: NC (hotel parisien independant) | CA: NC | Salaire: NC | Source: Journal des Palaces | Lien: https://www.journaldespalaces.com/carriere/offre-316727-Chef-de-reception-Hotel-L-Ormaie-Paris.html | Contexte: Hotel parisien independant (hors chaine) recrutant un chef de reception en CDI : encadrement d'une equipe front office, poste de management intermediaire.</t>
         </is>
       </c>
     </row>
@@ -2750,7 +2750,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Le Burgundy Paris</t>
+          <t>Hotel L'Ormaie</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -2766,12 +2766,12 @@
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>HOSPITALITY,JOB,DRH,50-200,CONTACT_2,CONTACT_NON_SOURCE</t>
+          <t>HOSPITALITY,JOB,DRH,5-50,CONTACT_2,CONTACT_NON_SOURCE</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Poste: Concierge (CDI) | Date: NC | Effectif: NC (hotel 5* independant, 59 chambres) | CA: NC | Salaire: NC | Source: Journal des Palaces | Lien: https://www.journaldespalaces.com/carriere/offre-318382-Concierge-Le-Burgundy-Paris.html | Contexte: Hotel 5* parisien independant (rue Duphot, Paris 1er). Recrutement d'un concierge en CDI, offre la plus recente du flux Journal des Palaces consultee.</t>
+          <t>Poste: Chef de reception (CDI) | Date: NC - offre active, ID 316727 (anteriorite probable &gt; 7 jours, a revalider) | Effectif: NC (hotel parisien independant) | CA: NC | Salaire: NC | Source: Journal des Palaces | Lien: https://www.journaldespalaces.com/carriere/offre-316727-Chef-de-reception-Hotel-L-Ormaie-Paris.html | Contexte: Hotel parisien independant (hors chaine) recrutant un chef de reception en CDI : encadrement d'une equipe front office, poste de management intermediaire.</t>
         </is>
       </c>
     </row>

</xml_diff>